<commit_message>
Fix wording in every pack, deck and tracker
</commit_message>
<xml_diff>
--- a/tutor-time/the-week-sheet/downloads/The_Week_Sheet.xlsx
+++ b/tutor-time/the-week-sheet/downloads/The_Week_Sheet.xlsx
@@ -111,13 +111,13 @@
     <t xml:space="preserve">A spare for next week</t>
   </si>
   <si>
-    <t xml:space="preserve">Fill in the shaded cells. Nobody marks this and nobody collects it in, so keep what actually happened on it: do not delete a session that got missed, move it into a spare and leave the old one where it was.</t>
+    <t xml:space="preserve">Fill in the shaded cells. Nobody marks this or collects it in. If a session gets missed, do not delete it: add “(moved to …)” after it and copy it into the next spare.</t>
   </si>
   <si>
     <t xml:space="preserve">A week that did not go to plan</t>
   </si>
   <si>
-    <t xml:space="preserve">One student’s week at the end of a real one. Two sessions moved, nothing was abandoned, and the three lines underneath are what makes the next week better.</t>
+    <t xml:space="preserve">One student’s sheet at the end of a real week. Two sessions moved, nothing was abandoned, and the three lines underneath are what makes the next week better.</t>
   </si>
   <si>
     <t xml:space="preserve">Chemistry: the six equations on the cards</t>

</xml_diff>